<commit_message>
New class & method add
</commit_message>
<xml_diff>
--- a/src/test/resources/LoginData.xlsx
+++ b/src/test/resources/LoginData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="46">
   <si>
     <t>Password</t>
   </si>
@@ -103,9 +103,6 @@
   </si>
   <si>
     <t>Male1</t>
-  </si>
-  <si>
-    <t>Female1</t>
   </si>
   <si>
     <t>ActData</t>
@@ -595,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -606,7 +603,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -617,7 +614,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -628,7 +625,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -655,7 +652,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -666,29 +663,29 @@
         <v>123456</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="3">
         <v>123456</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" s="3">
         <v>123456</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -696,10 +693,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -759,7 +756,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>14</v>
@@ -805,7 +802,7 @@
         <v>22</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>14</v>
@@ -859,7 +856,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
@@ -880,7 +877,7 @@
         <v>10</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -906,7 +903,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
@@ -932,7 +929,7 @@
         <v>19</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -952,13 +949,13 @@
         <v>22</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -984,7 +981,7 @@
         <v>19</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1009,10 +1006,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1041,13 +1038,13 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3"/>
     </row>
@@ -1066,7 +1063,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1076,7 +1073,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -1086,7 +1083,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>